<commit_message>
fix: remove PDF button and replace download file with exact user application Excel form
</commit_message>
<xml_diff>
--- a/public/2026_GTA_Application_form.xlsx
+++ b/public/2026_GTA_Application_form.xlsx
@@ -1,19 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
-  <bookViews>
-    <workbookView firstSheet="1" activeTab="1"/>
-  </bookViews>
+  <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1" state="hidden"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="ENG" sheetId="2" r:id="rId2"/>
     <sheet name="KOR" sheetId="3" r:id="rId3"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">ENG!$A$1:$Z$39</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">KOR!$A$1:$Z$35</definedName>
-  </definedNames>
 </workbook>
 </file>
 
@@ -695,7 +688,6 @@
     <mergeCell ref="A8:D8"/>
     <mergeCell ref="A9:D9"/>
   </mergeCells>
-  <pageMargins left="0.5118110236220472" right="0.5118110236220472" top="0.7480314960629921" bottom="0.7480314960629921" header="0.31496062992125984" footer="0.31496062992125984"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:AA37"/>
   </ignoredErrors>
@@ -704,7 +696,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA38"/>
+  <dimension ref="A1:Z38"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -987,16 +979,15 @@
     <mergeCell ref="B29:Q29"/>
     <mergeCell ref="B30:N30"/>
   </mergeCells>
-  <pageMargins left="0.7086614173228347" right="0.5118110236220472" top="0.7480314960629921" bottom="0.7480314960629921" header="0.31496062992125984" footer="0.31496062992125984"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AA38"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z38"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA35"/>
+  <dimension ref="A1:X35"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1237,9 +1228,8 @@
     <mergeCell ref="R30:Z30"/>
     <mergeCell ref="A32:Y32"/>
   </mergeCells>
-  <pageMargins left="0.7086614173228347" right="0.5118110236220472" top="0.7480314960629921" bottom="0.7480314960629921" header="0.31496062992125984" footer="0.31496062992125984"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AA35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:X35"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>